<commit_message>
Incorpora link apertura directa brochure proyecto 16-04-2026
</commit_message>
<xml_diff>
--- a/Proyectos/Proyectos.xlsx
+++ b/Proyectos/Proyectos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AI\cotizador-web-mp\Proyectos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1466F369-0EB8-4162-8A94-241C61F0253A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAD9981A-A7C3-4B22-B3F3-EE42FBF06955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{835DC9D8-6857-4F21-A726-3C93CCAB3C03}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="108">
   <si>
     <t>PROYECTO</t>
   </si>
@@ -345,13 +345,31 @@
   </si>
   <si>
     <t>https://drive.google.com/drive/folders/1LTL0Rttjnn8BLMCNyOhXScMODbuC0hUA?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1o72s8BBxu9_TSvA4N-9tzHER7CKI0OOI/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>LINK_PDF</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1QS_BqPDFeFyWkM2t_oeVENFJyDm4HS5i/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1rDI4XS2rIHtQJktqmVm8FMbrMrL4ikem/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1gNEj6Zv05PVaE7BmjRyd2nPVnLhGVDZq/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1XR3fasST9Di4ssakxugt9_rnDL7ysDga/view?usp=drive_link</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -375,6 +393,14 @@
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -574,10 +600,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -591,8 +618,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -927,7 +958,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52296A6F-29CA-48E9-B71C-2F11E9C03F57}">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.77734375" bestFit="1" customWidth="1"/>
@@ -935,9 +966,10 @@
     <col min="3" max="3" width="13.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="82.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -953,8 +985,11 @@
       <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" s="13" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
@@ -970,8 +1005,11 @@
       <c r="E2" s="8" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
@@ -987,8 +1025,11 @@
       <c r="E3" s="8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F3" s="14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>14</v>
       </c>
@@ -1004,8 +1045,11 @@
       <c r="E4" s="8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F4" s="15" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>17</v>
       </c>
@@ -1021,8 +1065,11 @@
       <c r="E5" s="8" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5" s="14" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>21</v>
       </c>
@@ -1038,8 +1085,11 @@
       <c r="E6" s="8" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F6" s="14" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>24</v>
       </c>
@@ -1056,7 +1106,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>27</v>
       </c>
@@ -1073,7 +1123,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>27</v>
       </c>
@@ -1090,7 +1140,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>31</v>
       </c>
@@ -1107,7 +1157,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>34</v>
       </c>
@@ -1124,7 +1174,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>37</v>
       </c>
@@ -1141,7 +1191,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>40</v>
       </c>
@@ -1158,7 +1208,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>42</v>
       </c>
@@ -1171,7 +1221,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>44</v>
       </c>
@@ -1184,7 +1234,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>46</v>
       </c>
@@ -1582,6 +1632,11 @@
     <hyperlink ref="E37" r:id="rId36" xr:uid="{12E413BB-BC88-480D-AF82-4C8DE4DF4CB2}"/>
     <hyperlink ref="E38" r:id="rId37" xr:uid="{916985DD-FEC6-41C1-A9D6-A9E6DFF473E1}"/>
     <hyperlink ref="E39" r:id="rId38" xr:uid="{459188E0-53E1-4DF8-868B-F349F2418CC9}"/>
+    <hyperlink ref="F2" r:id="rId39" xr:uid="{A14886E3-7086-448A-932B-0617C9E67B6B}"/>
+    <hyperlink ref="F3" r:id="rId40" xr:uid="{81144A1A-548C-4539-A749-1677BAA0E1B9}"/>
+    <hyperlink ref="F4" r:id="rId41" xr:uid="{21638768-309B-413F-908B-45831434D749}"/>
+    <hyperlink ref="F5" r:id="rId42" xr:uid="{31E4C781-CF33-4106-85CF-E142FFDCD240}"/>
+    <hyperlink ref="F6" r:id="rId43" xr:uid="{00F13436-D414-4435-9ABE-D66824AE730D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>